<commit_message>
Changes in python script and update of source templates for all nodes
</commit_message>
<xml_diff>
--- a/source/CSU/GF_CSU.xlsx
+++ b/source/CSU/GF_CSU.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/a1234414/Desktop/TEAMS/GF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C27F6EFE-5E24-E04D-9E8E-69F79320DE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C2EFFDA-5B64-4B16-9018-B9F050F277C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30040" yWindow="11560" windowWidth="26840" windowHeight="15760" firstSheet="1" activeTab="1" xr2:uid="{70CB10A7-9494-6A43-A40D-94D71C9EE1D6}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
-    <sheet name="growth facility list" sheetId="1" r:id="rId2"/>
+    <sheet name="growth facility" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -72,6 +72,42 @@
     <t>For any questions, please contact Liliana Andres at liliana.andreshernandez@adelaide.edu.au.</t>
   </si>
   <si>
+    <t>organisation</t>
+  </si>
+  <si>
+    <t>growth facility name *</t>
+  </si>
+  <si>
+    <t>growth facility description *</t>
+  </si>
+  <si>
+    <t>growth facility type *</t>
+  </si>
+  <si>
+    <t>growth facility type brand *</t>
+  </si>
+  <si>
+    <t>growth facility model *</t>
+  </si>
+  <si>
+    <t>growth facility serial number *</t>
+  </si>
+  <si>
+    <t>containment level *</t>
+  </si>
+  <si>
+    <t>quarantine details *</t>
+  </si>
+  <si>
+    <t>growth facility ontology label</t>
+  </si>
+  <si>
+    <t>growth facility ontology ID</t>
+  </si>
+  <si>
+    <t>growth facility ontology IRI</t>
+  </si>
+  <si>
     <t>CSU</t>
   </si>
   <si>
@@ -79,49 +115,13 @@
   </si>
   <si>
     <t>core 1</t>
-  </si>
-  <si>
-    <t>organization</t>
-  </si>
-  <si>
-    <t>growth facility name *</t>
-  </si>
-  <si>
-    <t>growth facility description *</t>
-  </si>
-  <si>
-    <t>growth facility type *</t>
-  </si>
-  <si>
-    <t>growth facility type brand *</t>
-  </si>
-  <si>
-    <t>growth facility model *</t>
-  </si>
-  <si>
-    <t>growth facility serial number *</t>
-  </si>
-  <si>
-    <t>containment level *</t>
-  </si>
-  <si>
-    <t>quarantine *</t>
-  </si>
-  <si>
-    <t>growth facility ontology label</t>
-  </si>
-  <si>
-    <t>growth facility ontology ID</t>
-  </si>
-  <si>
-    <t>growth facility ontology IRI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="13">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -130,13 +130,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -149,12 +142,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FF333F48"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -170,13 +157,6 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
@@ -213,24 +193,17 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color rgb="FF000000"/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="14"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -304,49 +277,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -698,62 +664,62 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA5B5531-C33C-4D11-A867-7D17CEB6AAAE}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="143.1640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" style="9" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" style="9" customWidth="1"/>
-    <col min="4" max="16384" width="9" style="9"/>
+    <col min="1" max="1" width="143.125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="18.375" style="6" customWidth="1"/>
+    <col min="3" max="3" width="25.875" style="6" customWidth="1"/>
+    <col min="4" max="16384" width="9" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:3" ht="26.1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="8"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="5"/>
     </row>
-    <row r="2" spans="1:3" ht="44" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:3" ht="44.1">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="10"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="7"/>
     </row>
-    <row r="3" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
-      <c r="C3" s="10"/>
+    <row r="3" spans="1:3" ht="21">
+      <c r="A3" s="10"/>
+      <c r="C3" s="7"/>
     </row>
-    <row r="4" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A4" s="13"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
+    <row r="4" spans="1:3" ht="21">
+      <c r="A4" s="10"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
     </row>
-    <row r="5" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:3" ht="21">
+      <c r="A5" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="10"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="7"/>
     </row>
-    <row r="6" spans="1:3" ht="44" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:3" ht="44.1">
+      <c r="A6" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
     </row>
-    <row r="7" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+    <row r="7" spans="1:3" ht="21">
+      <c r="A7" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
     </row>
-    <row r="8" spans="1:3" ht="21" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
+    <row r="8" spans="1:3" ht="21">
+      <c r="A8" s="11"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -762,64 +728,63 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85A53E4F-D382-9040-83D5-C82D41719DD3}">
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="37.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr defaultColWidth="37.5" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="9" max="9" width="31.6640625" customWidth="1"/>
+    <col min="9" max="9" width="31.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="6" customFormat="1" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" s="3" customFormat="1" ht="18.75">
+      <c r="A1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="E1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="F1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="G1" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="H1" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="I1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="J1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="K1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I1" s="19" t="s">
+      <c r="L1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:12" s="1" customFormat="1" ht="15.95">
+      <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="C2" s="12"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:12" ht="15.75" customHeight="1">
+      <c r="B3" t="s">
         <v>19</v>
-      </c>
-      <c r="M1" s="1"/>
-    </row>
-    <row r="2" spans="1:13" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="3"/>
-    </row>
-    <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -829,6 +794,32 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c57c0e25-d6d6-4f5b-b0b2-7d758d7a4949">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Image xmlns="c57c0e25-d6d6-4f5b-b0b2-7d758d7a4949" xsi:nil="true"/>
+    <TaxCatchAll xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23" xsi:nil="true"/>
+    <l544f18d430f4c0886024d9e622455c4 xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </l544f18d430f4c0886024d9e622455c4>
+    <jbe33349d2e04ad58f3e9557e0157918 xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </jbe33349d2e04ad58f3e9557e0157918>
+    <f876555452e44e5798dee990952b63ae xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </f876555452e44e5798dee990952b63ae>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="d560fd02-aa12-447b-bf2e-34c9e57d035a" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -837,7 +828,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007EE926928A949E41B5C68441ED11B2EA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="52be21af1a8349f18767d387bddd8232">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b2ccdccd-44c9-4047-9c28-347bfbb7eb23" xmlns:ns3="c57c0e25-d6d6-4f5b-b0b2-7d758d7a4949" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="10d9f1abffa380d50643d816c40c845c" ns2:_="" ns3:_="">
     <xsd:import namespace="b2ccdccd-44c9-4047-9c28-347bfbb7eb23"/>
@@ -1092,54 +1083,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c57c0e25-d6d6-4f5b-b0b2-7d758d7a4949">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Image xmlns="c57c0e25-d6d6-4f5b-b0b2-7d758d7a4949" xsi:nil="true"/>
-    <TaxCatchAll xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23" xsi:nil="true"/>
-    <l544f18d430f4c0886024d9e622455c4 xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </l544f18d430f4c0886024d9e622455c4>
-    <jbe33349d2e04ad58f3e9557e0157918 xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </jbe33349d2e04ad58f3e9557e0157918>
-    <f876555452e44e5798dee990952b63ae xmlns="b2ccdccd-44c9-4047-9c28-347bfbb7eb23">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </f876555452e44e5798dee990952b63ae>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="d560fd02-aa12-447b-bf2e-34c9e57d035a" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00F3C37E-118E-41FF-A564-7C83D79BE885}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10A3AE5-B648-4C4B-8990-1A6CA2E96FFD}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03520EE7-F521-42DD-B6B5-99CACC0DEA06}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00F3C37E-118E-41FF-A564-7C83D79BE885}"/>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1F90AB4-ED8E-4921-A877-4CFAEB8F7C64}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10A3AE5-B648-4C4B-8990-1A6CA2E96FFD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="506c2a08-141f-4590-812e-37f0e9140889"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{03520EE7-F521-42DD-B6B5-99CACC0DEA06}"/>
 </file>
</xml_diff>